<commit_message>
feat(P6): P6.xlsx 6-섹션 표준 구조 착수 + Dictionary 동반 성장
P6.xlsx를 DOH Standard로 리팩토링 시작. 산출물은 Excel(단일 원본)만 유지.

P6.xlsx (신규)
- 28개 Feature 전수 등재 (ID/EN/한글/Object/Attribute)
- 고정 6섹션: 정의 / 원인 추정 / 이후 나타날 가능성 / Strong Co-occurrence
  / 추가 검증 포인트 / 사고확장
- 'Observation' 항목 폐기 (Feature 자체가 Observation)
- 원인·결과 체인은 Mechanism M-ID로 통일 표기
- 대표 3종 표준화 완료: pelvis_open_early, early_extension, high_hands
  (나머지 25종 pending — 동일 패턴으로 순차 진행)
- '표준 규칙' 시트: 항목 구분 기준(원인/결과/Strong Co-occurrence) + Mechanism 표기 규칙

Dictionary 동반 성장 (Feature↔Dictionary 공진화)
- Mechanism_Dictionary: +2 (M-ROT-12 Trail Leg Drive, M-ROT-13 Body Rotation Leads) → 51
- Feature_Dictionary: +14 (referenced→feature 승격 및 신규 P6 Feature) → 29
- 재분류 반영: Arm Drop Insufficient(원인→결과), Head Elevation(원인/동반 혼용 정리)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/Feature_Dictionary.xlsx
+++ b/Feature_Dictionary.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Rename Log" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$J$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1310,8 +1310,660 @@
       </c>
       <c r="J16" s="3" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>deep_hands</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Deep Hands</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>손 깊음</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Hands</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Position/Depth</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전 대비 손이 정상보다 깊은(몸 뒤쪽) 위치에 있는 상대 위치 현상.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>referenced→feature 승격</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>shallow_hands</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Shallow Hands</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>손 얕음</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Hands</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Position/Depth</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Shallow</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전 대비 손이 정상보다 얕은(몸 앞쪽) 위치에 있는 상대 위치 현상.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>forward_hands</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Forward Hands</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>손 전방</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Hands</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Position/Direction</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Forward</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손이 정상보다 목표 방향(전방)으로 이동해 있는 상대 위치 현상.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>hands_too_far_from_body</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hands Too Far From Body</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>손이 몸에서 멀어짐</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Hands</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Far</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손과 몸통 사이 거리가 정상보다 먼 현상.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>hands_too_close_to_body</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Hands Too Close To Body</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>손이 몸에 가까움</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hands</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손과 몸통 사이 거리가 정상보다 가까운 현상.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>late_arm</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Late Arm</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>팔 하강 지연</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Timing</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Late</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전 진행 대비 팔의 하강·전달이 정상보다 지연된 현상.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>trail_elbow_behind_body</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Trail Elbow Behind Body</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>트레일 팔꿈치 뒤처짐</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Trail Elbow</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 트레일 팔꿈치가 흉곽보다 뒤(트레일측)에 남아있는 현상.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>M-ARM-05와 연결</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>steep_shaft</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Steep Shaft</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>가파른 샤프트</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Angle/Plane</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Steep</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 가파른 현상.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>referenced→feature 승격 (M-CLB-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>shallow_shaft</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Shallow Shaft</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>눕는 샤프트</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Angle/Plane</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Shallow</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 눕는 현상.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>referenced→feature 승격</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>casting</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Casting</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>캐스팅</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Cast</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손목 코킹 각(래그)이 조기에 풀리며 클럽이 일찍 펴지는 현상.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>M-CLB-01/05 연결</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>lead_pressure_insufficient</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Insufficient</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>리드측 압력 부족</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Location/Magnitude</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Lead·Insufficient</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 리드측 지면압력이 정상보다 부족한 현상.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>referenced→feature 승격 (M-PRS-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>lead_pressure_excessive</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>리드측 압력 과다</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Location/Magnitude</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Lead·Excessive</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 리드측 지면압력이 정상보다 과도한 현상.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>M-PRS-05 연결</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>incomplete_pressure_transfer</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Incomplete Pressure Transfer</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>압력 이동 미완성</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Timing</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Late</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 트레일→리드 압력 이동이 임팩트 전까지 완성되지 않는 현상.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>M-PRS-03 연결. Late Pressure Shift와 관계 검토</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>spin_out</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Spin-out</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>스핀아웃</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Pelvis</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Spin-out</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반이 트레일측 축으로 과회전하며 체중이동·시퀀스·클럽 전달이 함께 무너지는 복합 현상. 단순 과회전(Pelvis Rotation Excessive)과 구분.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>referenced→feature 승격 (M-ROT-09)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J16"/>
+  <autoFilter ref="A1:J30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
refactor: Observation_Dictionary 제거 + Feature_Dictionary 스키마 단순화
Feature = Observation 결론에 따라 Dictionary를 하나로 통합.
두 개 유지 시 Observation/Feature 경계가 모호해지는 문제 제거.

- 삭제: Observation_Dictionary.xlsx (Feature_Dictionary로 일원화)
- Feature_Dictionary.xlsx Features 시트 컬럼 단순화:
  Feature명 · 한글명 · 정의 · Category · 비고
  · Category = Object(분절: Pelvis/Thorax/Head/Hands/Arm/Shaft/Club/Pressure/Spine)
  · Attribute·상태·rename 등은 비고로 정리
- 참조 시트(Naming Rule / Controlled Vocabulary / Rename Log)는 표준 근거로 유지

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/Feature_Dictionary.xlsx
+++ b/Feature_Dictionary.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Rename Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$E$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,526 +469,318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Feature ID</t>
+          <t>Feature명</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Feature Name (EN)</t>
+          <t>한글명</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>한글명</t>
+          <t>정의</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Object</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Attribute Axis</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>정의</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>비고</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>pelvis_open_early</t>
+          <t>Pelvis Open Early</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Pelvis Open Early</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
           <t>골반 조기 오픈</t>
         </is>
       </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반이 정상보다 이른 타이밍에 목표 방향으로 열리는 현상. 회전량(Amount)이 아니라 회전 시점(Timing)의 문제가 핵심이다.</t>
+        </is>
+      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Timing</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Early</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반이 정상보다 이른 타이밍에 목표 방향으로 열리는 현상. 회전량(Amount)이 아니라 회전 시점(Timing)의 문제가 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>[구분] pelvis_rotation_excessive (회전량); pelvis_stall (회전 속도)</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Timing · Early
+[구분] pelvis_rotation_excessive (회전량); pelvis_stall (회전 속도)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>pelvis_rotation_insufficient</t>
+          <t>Pelvis Rotation Insufficient</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pelvis Rotation Insufficient</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
           <t>골반 회전 부족</t>
         </is>
       </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반의 회전량이 정상보다 부족한 현상. 회전 시점이나 속도가 아니라 회전량(Amount)이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Amount</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Insufficient</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반의 회전량이 정상보다 부족한 현상. 회전 시점이나 속도가 아니라 회전량(Amount)이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>[구분] thorax_rotation_insufficient (분절이 다름)</t>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Amount · Insufficient
+[구분] thorax_rotation_insufficient (분절이 다름)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>pelvis_rotation_excessive</t>
+          <t>Pelvis Rotation Excessive</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pelvis Rotation Excessive</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
           <t>골반 과회전</t>
         </is>
       </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반의 회전량이 정상보다 과도한 현상. 회전량만 많은 상태이며, 시퀀스·체중이동·클럽 전달까지 무너진 복합 현상인 Spin-out과는 구분한다.</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Amount</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Excessive</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반의 회전량이 정상보다 과도한 현상. 회전량만 많은 상태이며, 시퀀스·체중이동·클럽 전달까지 무너진 복합 현상인 Spin-out과는 구분한다.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>[구분] spin_out (회전량+시퀀스 붕괴 복합); pelvis_open_early (타이밍)</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Amount · Excessive
+[구분] spin_out (회전량+시퀀스 붕괴 복합); pelvis_open_early (타이밍)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>pelvis_stall</t>
+          <t>Pelvis Stall</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Pelvis Stall</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
           <t>골반 회전 정지</t>
         </is>
       </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반 회전이 정상보다 일찍 감속하거나 정지하는 현상. 회전량이 아니라 회전 속도(Velocity)가 유지되지 못하는 것이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Velocity</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Stall</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반 회전이 정상보다 일찍 감속하거나 정지하는 현상. 회전량이 아니라 회전 속도(Velocity)가 유지되지 못하는 것이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>[strong co-occur] handle_stall (선후 개인차, 양방향 연관 가능)</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Velocity · Stall
+[strong co-occur] handle_stall (선후 개인차, 양방향 연관 가능)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>thorax_rotation_insufficient</t>
+          <t>Thorax Rotation Insufficient</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Thorax Rotation Insufficient</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
           <t>흉곽 회전 부족</t>
         </is>
       </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽의 회전량이 정상보다 부족한 상태. 골반 회전과는 별개 Feature이며 상체 회전량(Amount) 부족이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Amount</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Insufficient</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 흉곽의 회전량이 정상보다 부족한 상태. 골반 회전과는 별개 Feature이며 상체 회전량(Amount) 부족이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Amount · Insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>thorax_rotation_excessive</t>
+          <t>Thorax Rotation Excessive</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Thorax Rotation Excessive</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
           <t>흉곽 과회전</t>
         </is>
       </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽의 회전량이 정상보다 과도한 상태. 회전 타이밍이 아니라 회전량(Amount)이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Amount</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Excessive</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 흉곽의 회전량이 정상보다 과도한 상태. 회전 타이밍이 아니라 회전량(Amount)이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Amount · Excessive</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>thorax_stall</t>
+          <t>Thorax Stall</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Thorax Stall</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
           <t>흉곽 회전 정지</t>
         </is>
       </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽 회전이 정상보다 일찍 감속하거나 정지하는 현상. 회전량이 아니라 회전 속도(Velocity) 유지 실패가 핵심이다.</t>
+        </is>
+      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Velocity</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Stall</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 흉곽 회전이 정상보다 일찍 감속하거나 정지하는 현상. 회전량이 아니라 회전 속도(Velocity) 유지 실패가 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>[strong co-occur] pelvis_stall (선후 개인차)</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Velocity · Stall
+[strong co-occur] pelvis_stall (선후 개인차)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>thorax_open_early</t>
+          <t>Thorax Open Early</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Thorax Open Early</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
           <t>흉곽 조기 오픈</t>
         </is>
       </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 흉곽이 정상보다 이른 타이밍에 목표 방향으로 열리는 현상. 회전량이 아니라 회전 시점(Timing)이 빠른 것이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Thorax</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Rotation/Timing</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Early</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 흉곽이 정상보다 이른 타이밍에 목표 방향으로 열리는 현상. 회전량이 아니라 회전 시점(Timing)이 빠른 것이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>[renamed from] Upper Body Open Early</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Rotation/Timing · Early
+[renamed from] Upper Body Open Early</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>early_extension</t>
+          <t>Early Extension</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Early Extension</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
           <t>얼리 익스텐션</t>
         </is>
       </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반이 볼 방향으로 전진하거나 고관절 굴곡이 조기에 소실되면서 몸이 일찍 일어나는 현상. 골반·고관절·척추 자세를 유지하지 못하고 신체가 조기에 신전되는 것이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Pattern</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Early Extension</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반이 볼 방향으로 전진하거나 고관절 굴곡이 조기에 소실되면서 몸이 일찍 일어나는 현상. 골반·고관절·척추 자세를 유지하지 못하고 신체가 조기에 신전되는 것이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>[role] Hub Node — 다수 원인이 모이고 다수 결과로 분기. In/Out-degree 모두 높음.</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Pattern · Early Extension
+[role] Hub Node — 다수 원인이 모이고 다수 결과로 분기. In/Out-degree 모두 높음.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>spine_extension_excessive</t>
+          <t>Spine Extension Excessive</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Spine Extension Excessive</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
           <t>척추 과신전</t>
         </is>
       </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 척추(흉요추)가 정상보다 과도하게 신전되어 상체가 뒤로 젖는 현상. 평가 분절이 골반/고관절인 Early Extension과 구분한다.</t>
+        </is>
+      </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Spine</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Magnitude</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Excessive</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 척추(흉요추)가 정상보다 과도하게 신전되어 상체가 뒤로 젖는 현상. 평가 분절이 골반/고관절인 Early Extension과 구분한다.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>[renamed from] Excessive Spine Extension
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Magnitude · Excessive
+[renamed from] Excessive Spine Extension
 [구분] early_extension (분절: 골반/고관절)</t>
         </is>
       </c>
@@ -996,47 +788,28 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>head_elevation</t>
+          <t>Head Elevation</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Head Elevation</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
           <t>머리 상승</t>
         </is>
       </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 머리 높이가 정상보다 상승하는 현상. 목만이 아니라 몸 전체의 수직 움직임/자세 변화로 머리가 위로 이동하는 것이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Position/Height (Vertical Axis)</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Rise</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 머리 높이가 정상보다 상승하는 현상. 목만이 아니라 몸 전체의 수직 움직임/자세 변화로 머리가 위로 이동하는 것이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>[role] Result Feature 성격 강함 — In-degree 높음.
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Position/Height (Vertical Axis) · Rise
+[role] Result Feature 성격 강함 — In-degree 높음.
 [phase] P6에서는 초기 발생, P7에서 최종 관찰되는 경우가 많음. 두 구간 체크 대상.</t>
         </is>
       </c>
@@ -1044,843 +817,507 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>head_drop</t>
+          <t>Head Drop</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Head Drop</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
           <t>머리 하강</t>
         </is>
       </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 머리 높이가 정상보다 과도하게 낮아지는 현상. 정상적 지면반응·측굴에 의한 자연스러운 하강이 아니라 상체가 숙여지며 머리가 낮아지는 것이 핵심이다.</t>
+        </is>
+      </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Position/Height (Vertical Axis)</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Drop</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 머리 높이가 정상보다 과도하게 낮아지는 현상. 정상적 지면반응·측굴에 의한 자연스러운 하강이 아니라 상체가 숙여지며 머리가 낮아지는 것이 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>[구분] head_elevation (단순 ± 관계 아님 — 원인·결과 Chain 상이)</t>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Position/Height (Vertical Axis) · Drop
+[구분] head_elevation (단순 ± 관계 아님 — 원인·결과 Chain 상이)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>head_hanging_back</t>
+          <t>Head Hanging Back</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Head Hanging Back</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
           <t>머리 뒤잔류</t>
         </is>
       </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 머리 위치가 정상보다 후방(트레일측)에 남아 목표 방향으로 이동하지 못하는 현상. 체중 패턴(Hanging Back)과는 별개의 머리 위치 Feature이다.</t>
+        </is>
+      </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Position/Location (Horizontal Axis)</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Trail</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 머리 위치가 정상보다 후방(트레일측)에 남아 목표 방향으로 이동하지 못하는 현상. 체중 패턴(Hanging Back)과는 별개의 머리 위치 Feature이다.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>[구분] hanging_back (체중 패턴)</t>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Position/Location (Horizontal Axis) · Trail
+[구분] hanging_back (체중 패턴)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>high_hands</t>
+          <t>High Hands</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>High Hands</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
           <t>손 높음</t>
         </is>
       </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Position/Height (Relative)</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 높은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 충분히 하강하지 못한 상대 위치가 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Position/Height (Relative) · High</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>low_hands</t>
+          <t>Low Hands</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Low Hands</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
           <t>손 낮음</t>
         </is>
       </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 낮은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 과도하게 하강한 상대 위치가 핵심이다.</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Position/Height (Relative)</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전·다운스윙 진행 정도에 비해 손이 정상보다 낮은 위치에 있는 현상. 절대 높이가 아니라 몸의 회전 대비 손이 과도하게 하강한 상대 위치가 핵심이다.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Position/Height (Relative) · Low</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>deep_hands</t>
+          <t>Deep Hands</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Deep Hands</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
           <t>손 깊음</t>
         </is>
       </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전 대비 손이 정상보다 깊은(몸 뒤쪽) 위치에 있는 상대 위치 현상.</t>
+        </is>
+      </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Position/Depth</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Deep</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전 대비 손이 정상보다 깊은(몸 뒤쪽) 위치에 있는 상대 위치 현상.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Position/Depth · Deep
+[status] pending  ·  referenced→feature 승격</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>shallow_hands</t>
+          <t>Shallow Hands</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Shallow Hands</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
           <t>손 얕음</t>
         </is>
       </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전 대비 손이 정상보다 얕은(몸 앞쪽) 위치에 있는 상대 위치 현상.</t>
+        </is>
+      </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Position/Depth</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Shallow</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전 대비 손이 정상보다 얕은(몸 앞쪽) 위치에 있는 상대 위치 현상.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Position/Depth · Shallow
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>Forward Hands</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Forward Hands</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
           <t>손 전방</t>
         </is>
       </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손이 정상보다 목표 방향(전방)으로 이동해 있는 상대 위치 현상.</t>
+        </is>
+      </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Position/Direction</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Forward</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 손이 정상보다 목표 방향(전방)으로 이동해 있는 상대 위치 현상.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Position/Direction · Forward
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far_from_body</t>
+          <t>Hands Too Far From Body</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Hands Too Far From Body</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
           <t>손이 몸에서 멀어짐</t>
         </is>
       </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손과 몸통 사이 거리가 정상보다 먼 현상.</t>
+        </is>
+      </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Relationship</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Far</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 손과 몸통 사이 거리가 정상보다 먼 현상.</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Relationship · Far
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close_to_body</t>
+          <t>Hands Too Close To Body</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Hands Too Close To Body</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
           <t>손이 몸에 가까움</t>
         </is>
       </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손과 몸통 사이 거리가 정상보다 가까운 현상.</t>
+        </is>
+      </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Hands</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Relationship</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Close</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 손과 몸통 사이 거리가 정상보다 가까운 현상.</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Relationship · Close
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>late_arm</t>
+          <t>Late Arm</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Late Arm</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
           <t>팔 하강 지연</t>
         </is>
       </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 몸의 회전 진행 대비 팔의 하강·전달이 정상보다 지연된 현상.</t>
+        </is>
+      </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Arm</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Timing</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Late</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 몸의 회전 진행 대비 팔의 하강·전달이 정상보다 지연된 현상.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Timing · Late
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>trail_elbow_behind_body</t>
+          <t>Trail Elbow Behind Body</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Trail Elbow Behind Body</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
           <t>트레일 팔꿈치 뒤처짐</t>
         </is>
       </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 트레일 팔꿈치가 흉곽보다 뒤(트레일측)에 남아있는 현상.</t>
+        </is>
+      </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Trail Elbow</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Trail</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 트레일 팔꿈치가 흉곽보다 뒤(트레일측)에 남아있는 현상.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Location · Trail
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>steep_shaft</t>
+          <t>Steep Shaft</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Steep Shaft</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
           <t>가파른 샤프트</t>
         </is>
       </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 가파른 현상.</t>
+        </is>
+      </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Shaft</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Angle/Plane</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Steep</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 가파른 현상.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Angle/Plane · Steep
+[status] pending  ·  referenced→feature 승격</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>shallow_shaft</t>
+          <t>Shallow Shaft</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Shallow Shaft</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
           <t>눕는 샤프트</t>
         </is>
       </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 눕는 현상.</t>
+        </is>
+      </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Shaft</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Angle/Plane</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Shallow</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 샤프트 플레인이 정상보다 눕는 현상.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Angle/Plane · Shallow
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>casting</t>
+          <t>Casting</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Casting</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
           <t>캐스팅</t>
         </is>
       </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 손목 코킹 각(래그)이 조기에 풀리며 클럽이 일찍 펴지는 현상.</t>
+        </is>
+      </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Cast</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 손목 코킹 각(래그)이 조기에 풀리며 클럽이 일찍 펴지는 현상.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Release · Cast
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_insufficient</t>
+          <t>Lead Pressure Insufficient</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Lead Pressure Insufficient</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
           <t>리드측 압력 부족</t>
         </is>
       </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 리드측 지면압력이 정상보다 부족한 현상.</t>
+        </is>
+      </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Location/Magnitude</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Lead·Insufficient</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 리드측 지면압력이 정상보다 부족한 현상.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Location/Magnitude · Lead·Insufficient
+[status] pending  ·  referenced→feature 승격</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive</t>
+          <t>Lead Pressure Excessive</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Lead Pressure Excessive</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
           <t>리드측 압력 과다</t>
         </is>
       </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 리드측 지면압력이 정상보다 과도한 현상.</t>
+        </is>
+      </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Location/Magnitude</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Lead·Excessive</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 리드측 지면압력이 정상보다 과도한 현상.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Location/Magnitude · Lead·Excessive
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>incomplete_pressure_transfer</t>
+          <t>Incomplete Pressure Transfer</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Incomplete Pressure Transfer</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
           <t>압력 이동 미완성</t>
         </is>
       </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 트레일→리드 압력 이동이 임팩트 전까지 완성되지 않는 현상.</t>
+        </is>
+      </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Timing</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Late</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 트레일→리드 압력 이동이 임팩트 전까지 완성되지 않는 현상.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Timing · Late
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>spin_out</t>
+          <t>Spin-out</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Spin-out</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
           <t>스핀아웃</t>
         </is>
       </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>다운스윙 중반(P6)에서 골반이 트레일측 축으로 과회전하며 체중이동·시퀀스·클럽 전달이 함께 무너지는 복합 현상. 단순 과회전(Pelvis Rotation Excessive)과 구분.</t>
+        </is>
+      </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Pelvis</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Pattern</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Spin-out</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>다운스윙 중반(P6)에서 골반이 트레일측 축으로 과회전하며 체중이동·시퀀스·클럽 전달이 함께 무너지는 복합 현상.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>referenced→feature 승격</t>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Pattern · Spin-out
+[status] pending  ·  referenced→feature 승격</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
+  <autoFilter ref="A1:E30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1948,7 +1385,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Objects</t>
+          <t>Objects (= Category)</t>
         </is>
       </c>
     </row>

</xml_diff>